<commit_message>
Lab02, everything regarding tests has been added and 'Tested'
</commit_message>
<xml_diff>
--- a/docs/Lab01/Lab01_ReviewReport.xlsx
+++ b/docs/Lab01/Lab01_ReviewReport.xlsx
@@ -5,7 +5,7 @@
   <workbookPr backupFile="false" showObjects="all" dateCompatibility="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="1"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Requirements Phase Defects" sheetId="1" state="visible" r:id="rId3"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="65">
   <si>
     <t xml:space="preserve">do not print this form</t>
   </si>
@@ -70,13 +70,13 @@
     <t xml:space="preserve">Reviewer Name:</t>
   </si>
   <si>
-    <t xml:space="preserve">amandoi</t>
+    <t xml:space="preserve">Nuta Rafael si Onofrei Efraim</t>
   </si>
   <si>
     <t xml:space="preserve">Review date: </t>
   </si>
   <si>
-    <t xml:space="preserve">07.03.2025</t>
+    <t xml:space="preserve">07.03.2026</t>
   </si>
   <si>
     <t xml:space="preserve">Crt. No.</t>
@@ -173,6 +173,30 @@
   </si>
   <si>
     <t xml:space="preserve">Popescu Ionel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C01</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DrinkShopController.java</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Liniile 122 si 123, if else despartit in 2 linii separate</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C04</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linia 144, se parseaza textul fara a valida ca ar putea corespunde unui nr real</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C08</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linia 119, mesaj de eroare gresit: “adugati”</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linia 246, export-ul de date se face mereu in acelasi fisier hardcodat</t>
   </si>
   <si>
     <t xml:space="preserve">Tool-based Code Analysis</t>
@@ -203,7 +227,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="11">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -265,6 +289,12 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i val="true"/>
@@ -363,116 +393,120 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -825,22 +859,22 @@
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="E7" s="12"/>
+      <c r="E7" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="14" t="s">
+      <c r="E9" s="15" t="s">
         <v>21</v>
       </c>
     </row>
@@ -848,13 +882,13 @@
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="15" t="s">
+      <c r="D10" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="17" t="s">
         <v>24</v>
       </c>
     </row>
@@ -863,13 +897,13 @@
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D11" s="15" t="s">
+      <c r="D11" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>27</v>
       </c>
     </row>
@@ -878,13 +912,13 @@
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="16" t="s">
         <v>28</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="17" t="s">
         <v>29</v>
       </c>
     </row>
@@ -893,13 +927,13 @@
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="17" t="s">
         <v>32</v>
       </c>
     </row>
@@ -908,13 +942,13 @@
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15" t="s">
+      <c r="C14" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="D14" s="15" t="s">
+      <c r="D14" s="16" t="s">
         <v>31</v>
       </c>
-      <c r="E14" s="16" t="s">
+      <c r="E14" s="17" t="s">
         <v>33</v>
       </c>
     </row>
@@ -923,27 +957,27 @@
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="15"/>
-      <c r="E17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="16"/>
+      <c r="E17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
@@ -952,7 +986,7 @@
       </c>
       <c r="C18" s="6"/>
       <c r="D18" s="6"/>
-      <c r="E18" s="17"/>
+      <c r="E18" s="18"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
@@ -961,7 +995,7 @@
       </c>
       <c r="C19" s="6"/>
       <c r="D19" s="6"/>
-      <c r="E19" s="17"/>
+      <c r="E19" s="18"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
@@ -970,7 +1004,7 @@
       </c>
       <c r="C20" s="6"/>
       <c r="D20" s="6"/>
-      <c r="E20" s="17"/>
+      <c r="E20" s="18"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
@@ -979,7 +1013,7 @@
       </c>
       <c r="C21" s="6"/>
       <c r="D21" s="6"/>
-      <c r="E21" s="17"/>
+      <c r="E21" s="18"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
@@ -988,7 +1022,7 @@
       </c>
       <c r="C22" s="6"/>
       <c r="D22" s="6"/>
-      <c r="E22" s="17"/>
+      <c r="E22" s="18"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
@@ -997,7 +1031,7 @@
       </c>
       <c r="C23" s="6"/>
       <c r="D23" s="6"/>
-      <c r="E23" s="17"/>
+      <c r="E23" s="18"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
@@ -1006,7 +1040,7 @@
       </c>
       <c r="C24" s="6"/>
       <c r="D24" s="6"/>
-      <c r="E24" s="17"/>
+      <c r="E24" s="18"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
@@ -1015,14 +1049,14 @@
       </c>
       <c r="C25" s="6"/>
       <c r="D25" s="6"/>
-      <c r="E25" s="17"/>
+      <c r="E25" s="18"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C27" s="18" t="s">
+      <c r="C27" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D27" s="19"/>
-      <c r="E27" s="15" t="s">
+      <c r="D27" s="20"/>
+      <c r="E27" s="16" t="s">
         <v>35</v>
       </c>
     </row>
@@ -1093,31 +1127,39 @@
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="I3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="22" t="s">
         <v>37</v>
       </c>
-      <c r="E4" s="21"/>
+      <c r="E4" s="22"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
+      <c r="I4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="20" t="s">
+      <c r="C5" s="21" t="s">
         <v>38</v>
       </c>
-      <c r="D5" s="22" t="s">
+      <c r="D5" s="23" t="s">
         <v>39</v>
       </c>
-      <c r="E5" s="22"/>
+      <c r="E5" s="23"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1129,27 +1171,31 @@
       <c r="C6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="12"/>
+      <c r="D6" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="E6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="D7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>21</v>
       </c>
     </row>
@@ -1157,13 +1203,13 @@
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15" t="s">
+      <c r="C10" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="17" t="s">
         <v>42</v>
       </c>
     </row>
@@ -1172,13 +1218,13 @@
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="17" t="s">
         <v>41</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="17" t="s">
         <v>44</v>
       </c>
     </row>
@@ -1187,13 +1233,13 @@
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15" t="s">
+      <c r="C12" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D12" s="15" t="s">
+      <c r="D12" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E12" s="16" t="s">
+      <c r="E12" s="17" t="s">
         <v>45</v>
       </c>
     </row>
@@ -1202,13 +1248,13 @@
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15" t="s">
+      <c r="C13" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D13" s="15" t="s">
+      <c r="D13" s="16" t="s">
         <v>41</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="17" t="s">
         <v>46</v>
       </c>
     </row>
@@ -1217,124 +1263,124 @@
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="15"/>
-      <c r="E15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="16"/>
+      <c r="E15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="15"/>
-      <c r="E18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="16"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="16"/>
-      <c r="E19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="17"/>
+      <c r="E19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="15"/>
-      <c r="E20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="16"/>
+      <c r="E20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="15"/>
-      <c r="E22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="16"/>
+      <c r="E22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="15"/>
-      <c r="E23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="15"/>
-      <c r="E24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="16"/>
+      <c r="E24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="15"/>
-      <c r="E25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="16"/>
+      <c r="E25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C28" s="18" t="s">
+      <c r="C28" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D28" s="19"/>
-      <c r="E28" s="15"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1367,7 +1413,7 @@
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="8.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="12.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16.27"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="21.58"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="41.45"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="8" min="6" style="1" width="8.91"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="1" width="26.73"/>
@@ -1404,31 +1450,39 @@
       <c r="H3" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="6"/>
-      <c r="J3" s="6"/>
+      <c r="I3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="J3" s="6" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="23" t="s">
+      <c r="C4" s="24" t="s">
         <v>7</v>
       </c>
-      <c r="D4" s="24" t="s">
+      <c r="D4" s="25" t="s">
         <v>48</v>
       </c>
-      <c r="E4" s="24"/>
+      <c r="E4" s="25"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="I4" s="6"/>
-      <c r="J4" s="6"/>
+      <c r="I4" s="6" t="s">
+        <v>10</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>235</v>
+      </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="24" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="25" t="s">
+      <c r="D5" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="E5" s="25"/>
+      <c r="E5" s="26"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1440,224 +1494,252 @@
       <c r="C6" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D6" s="12"/>
+      <c r="D6" s="12" t="s">
+        <v>15</v>
+      </c>
       <c r="E6" s="12"/>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="C7" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D7" s="12"/>
-      <c r="E7" s="12"/>
+      <c r="D7" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="E7" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
+      <c r="C9" s="14" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="13" t="s">
+      <c r="D9" s="14" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="13" t="s">
+      <c r="E9" s="14" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" customFormat="false" ht="24.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-    </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C10" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D10" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E10" s="17" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="24.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="n">
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16"/>
+      <c r="C11" s="16" t="s">
+        <v>53</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="17" t="s">
+        <v>54</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="n">
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-    </row>
-    <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C12" s="16" t="s">
+        <v>55</v>
+      </c>
+      <c r="D12" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="17" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="24.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="n">
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
+      <c r="C13" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="D13" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="E13" s="17" t="s">
+        <v>57</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="n">
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="n">
         <f aca="false">B26+1</f>
         <v>18</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="15"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="n">
         <f aca="false">B27+1</f>
         <v>19</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="n">
         <f aca="false">B28+1</f>
         <v>20</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="n">
         <f aca="false">B29+1</f>
         <v>21</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="18" t="s">
+      <c r="C32" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D32" s="19"/>
-      <c r="E32" s="15"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="16"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -1711,7 +1793,7 @@
     </row>
     <row r="2" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B2" s="5" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="C2" s="5"/>
       <c r="D2" s="5"/>
@@ -1732,11 +1814,11 @@
       <c r="J3" s="6"/>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C4" s="23" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
+      <c r="C4" s="24" t="s">
+        <v>59</v>
+      </c>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
       <c r="H4" s="6" t="s">
         <v>9</v>
       </c>
@@ -1747,8 +1829,8 @@
       <c r="C5" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="12"/>
-      <c r="E5" s="12"/>
+      <c r="D5" s="13"/>
+      <c r="E5" s="13"/>
       <c r="H5" s="6" t="s">
         <v>13</v>
       </c>
@@ -1760,242 +1842,242 @@
       <c r="C6" s="11" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="12"/>
-      <c r="E6" s="12"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B9" s="13" t="s">
+      <c r="B9" s="14" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>53</v>
-      </c>
-      <c r="E9" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="F9" s="13" t="s">
-        <v>55</v>
+      <c r="C9" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="F9" s="14" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B10" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="16"/>
-      <c r="E10" s="16"/>
-      <c r="F10" s="16"/>
+      <c r="C10" s="16"/>
+      <c r="D10" s="17"/>
+      <c r="E10" s="17"/>
+      <c r="F10" s="17"/>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B11" s="6" t="n">
         <f aca="false">B10+1</f>
         <v>2</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="15"/>
-      <c r="E11" s="16"/>
-      <c r="F11" s="16"/>
+      <c r="C11" s="16"/>
+      <c r="D11" s="16"/>
+      <c r="E11" s="17"/>
+      <c r="F11" s="17"/>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B12" s="6" t="n">
         <f aca="false">B11+1</f>
         <v>3</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="15"/>
-      <c r="E12" s="16"/>
-      <c r="F12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="17"/>
+      <c r="F12" s="17"/>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="6" t="n">
         <f aca="false">B12+1</f>
         <v>4</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="16"/>
-      <c r="E13" s="16"/>
-      <c r="F13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="17"/>
+      <c r="E13" s="17"/>
+      <c r="F13" s="17"/>
     </row>
     <row r="14" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B14" s="6" t="n">
         <f aca="false">B13+1</f>
         <v>5</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="16"/>
-      <c r="E14" s="16"/>
-      <c r="F14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="D14" s="17"/>
+      <c r="E14" s="17"/>
+      <c r="F14" s="17"/>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="6" t="n">
         <f aca="false">B14+1</f>
         <v>6</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="16"/>
-      <c r="E15" s="16"/>
-      <c r="F15" s="16"/>
+      <c r="C15" s="16"/>
+      <c r="D15" s="17"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="17"/>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B16" s="6" t="n">
         <f aca="false">B15+1</f>
         <v>7</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="16"/>
-      <c r="E16" s="16"/>
-      <c r="F16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="17"/>
+      <c r="E16" s="17"/>
+      <c r="F16" s="17"/>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B17" s="6" t="n">
         <f aca="false">B16+1</f>
         <v>8</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="16"/>
-      <c r="E17" s="16"/>
-      <c r="F17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="17"/>
+      <c r="E17" s="17"/>
+      <c r="F17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="6" t="n">
         <f aca="false">B17+1</f>
         <v>9</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="16"/>
-      <c r="E18" s="16"/>
-      <c r="F18" s="16"/>
+      <c r="C18" s="16"/>
+      <c r="D18" s="17"/>
+      <c r="E18" s="17"/>
+      <c r="F18" s="17"/>
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="6" t="n">
         <f aca="false">B18+1</f>
         <v>10</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="15"/>
-      <c r="E19" s="16"/>
-      <c r="F19" s="16"/>
+      <c r="C19" s="16"/>
+      <c r="D19" s="16"/>
+      <c r="E19" s="17"/>
+      <c r="F19" s="17"/>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B20" s="6" t="n">
         <f aca="false">B19+1</f>
         <v>11</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="16"/>
-      <c r="E20" s="16"/>
-      <c r="F20" s="16"/>
+      <c r="C20" s="16"/>
+      <c r="D20" s="17"/>
+      <c r="E20" s="17"/>
+      <c r="F20" s="17"/>
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="6" t="n">
         <f aca="false">B20+1</f>
         <v>12</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="15"/>
-      <c r="E21" s="16"/>
-      <c r="F21" s="16"/>
+      <c r="C21" s="16"/>
+      <c r="D21" s="16"/>
+      <c r="E21" s="17"/>
+      <c r="F21" s="17"/>
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="6" t="n">
         <f aca="false">B21+1</f>
         <v>13</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="16"/>
-      <c r="E22" s="16"/>
-      <c r="F22" s="16"/>
+      <c r="C22" s="16"/>
+      <c r="D22" s="17"/>
+      <c r="E22" s="17"/>
+      <c r="F22" s="17"/>
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B23" s="6" t="n">
         <f aca="false">B22+1</f>
         <v>14</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="16"/>
-      <c r="E23" s="16"/>
-      <c r="F23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="17"/>
+      <c r="E23" s="17"/>
+      <c r="F23" s="17"/>
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B24" s="6" t="n">
         <f aca="false">B23+1</f>
         <v>15</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
-      <c r="F24" s="16"/>
+      <c r="C24" s="16"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
+      <c r="F24" s="17"/>
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B25" s="6" t="n">
         <f aca="false">B24+1</f>
         <v>16</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="16"/>
-      <c r="E25" s="16"/>
-      <c r="F25" s="16"/>
+      <c r="C25" s="16"/>
+      <c r="D25" s="17"/>
+      <c r="E25" s="17"/>
+      <c r="F25" s="17"/>
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B26" s="6" t="n">
         <f aca="false">B25+1</f>
         <v>17</v>
       </c>
-      <c r="C26" s="15"/>
-      <c r="D26" s="15"/>
-      <c r="E26" s="16"/>
-      <c r="F26" s="16"/>
+      <c r="C26" s="16"/>
+      <c r="D26" s="16"/>
+      <c r="E26" s="17"/>
+      <c r="F26" s="17"/>
     </row>
     <row r="27" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B27" s="6" t="n">
         <f aca="false">B26+1</f>
         <v>18</v>
       </c>
-      <c r="C27" s="15"/>
-      <c r="D27" s="16"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
+      <c r="C27" s="16"/>
+      <c r="D27" s="17"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B28" s="6" t="n">
         <f aca="false">B27+1</f>
         <v>19</v>
       </c>
-      <c r="C28" s="15"/>
-      <c r="D28" s="16"/>
-      <c r="E28" s="16"/>
-      <c r="F28" s="16"/>
+      <c r="C28" s="16"/>
+      <c r="D28" s="17"/>
+      <c r="E28" s="17"/>
+      <c r="F28" s="17"/>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B29" s="6" t="n">
         <f aca="false">B28+1</f>
         <v>20</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="16"/>
-      <c r="E29" s="16"/>
-      <c r="F29" s="16"/>
+      <c r="C29" s="16"/>
+      <c r="D29" s="17"/>
+      <c r="E29" s="17"/>
+      <c r="F29" s="17"/>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B30" s="6" t="n">
         <f aca="false">B29+1</f>
         <v>21</v>
       </c>
-      <c r="C30" s="15"/>
-      <c r="D30" s="16"/>
-      <c r="E30" s="16"/>
-      <c r="F30" s="16"/>
+      <c r="C30" s="16"/>
+      <c r="D30" s="17"/>
+      <c r="E30" s="17"/>
+      <c r="F30" s="17"/>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C32" s="26" t="s">
-        <v>56</v>
-      </c>
-      <c r="D32" s="26"/>
-      <c r="E32" s="26"/>
-      <c r="F32" s="27"/>
+      <c r="C32" s="27" t="s">
+        <v>64</v>
+      </c>
+      <c r="D32" s="27"/>
+      <c r="E32" s="27"/>
+      <c r="F32" s="28"/>
     </row>
   </sheetData>
   <mergeCells count="6">

</xml_diff>